<commit_message>
fix: 09-17 蓄積修正 — socio-rx サムネ / company-facts ロゴ二重 / seed-BL検証 / min_effective_chars / ログローテーション
- socio-rx サムネ「パス未指定」: monologue 分岐が short_thumbnail を返して
  いなかった。generate_short_thumbnail を呼ぶよう修正（失敗時も動画は続行）
- company-facts ロゴ二重表示: フォールバック背景の hero ロゴと logo_chip が
  同時に描かれていた。hero を敷いた回はチップを描かない
- seed-BL衝突の事前検証: config_validation に seed_blacklist_collision を追加。
  theme_seeds / autopilot.theme_queue を実運用と同じ blacklist_match で照合し
  読み込み時に警告。socio-rx キューの「久保建英」衝突1件を検出・除去
- min_effective_chars: 「なぜ〜のか」型（ch内対照 4/4ch・1.42x）に限り下限を
  20→15字へ緩和（一律引き下げは逆U字の実測と矛盾するため却下）。
  キュー違反 35→25件
- ログローテーション: scripts/rotate_backend_log.sh + launchd
  com.youtube-factory.logrotate（毎日04:30・20MB以上で copytruncate・7世代保持）。
  84MB の backend.log を初回ローテート済み
- 09-17 指揮者・PDCA のデータ更新と引き継ぎレポートを同梱

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reports/pdca_history.xlsx
+++ b/data/reports/pdca_history.xlsx
@@ -22,19 +22,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="socio-rx" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'daily-science'!$A$1:$O$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'scp-lab'!$A$1:$O$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'pokemon-lab'!$A$1:$O$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'yokai-watch'!$A$1:$O$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2ch-matome'!$A$1:$O$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'fake-paper'!$A$1:$O$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'akashic-librarian'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'clip-animal'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'clip-fukada'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'clip-kaneko'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'clip-lab'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'company-facts'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'socio-rx'!$A$1:$O$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'daily-science'!$A$1:$O$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'scp-lab'!$A$1:$O$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'pokemon-lab'!$A$1:$O$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'yokai-watch'!$A$1:$O$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2ch-matome'!$A$1:$O$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'fake-paper'!$A$1:$O$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'akashic-librarian'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'clip-animal'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'clip-fukada'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'clip-kaneko'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'clip-lab'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'company-facts'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'socio-rx'!$A$1:$O$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3995,8 +3995,122 @@
         <v>0</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>74</v>
+      </c>
+      <c r="C68" t="n">
+        <v>207053</v>
+      </c>
+      <c r="D68" t="n">
+        <v>220</v>
+      </c>
+      <c r="E68" t="n">
+        <v>45</v>
+      </c>
+      <c r="F68" t="n">
+        <v>912</v>
+      </c>
+      <c r="G68" t="n">
+        <v>952</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.6679</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>宇宙・天体</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>15</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>75</v>
+      </c>
+      <c r="C69" t="n">
+        <v>209387</v>
+      </c>
+      <c r="D69" t="n">
+        <v>224</v>
+      </c>
+      <c r="E69" t="n">
+        <v>48</v>
+      </c>
+      <c r="F69" t="n">
+        <v>916.7</v>
+      </c>
+      <c r="G69" t="n">
+        <v>953</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.6617</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>宇宙・天体</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>15</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O67"/>
+  <autoFilter ref="A1:O69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4007,7 +4121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4720,7 +4834,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>3</v>
       </c>
@@ -4738,8 +4851,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:O17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4750,7 +4950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5473,7 +5673,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -5491,8 +5690,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:O17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5503,7 +5789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6253,7 +6539,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -6271,8 +6556,113 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>42</v>
+      </c>
+      <c r="C16" t="n">
+        <v>65778</v>
+      </c>
+      <c r="D16" t="n">
+        <v>57</v>
+      </c>
+      <c r="E16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1210.8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1057</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.6012999999999999</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>42</v>
+      </c>
+      <c r="C17" t="n">
+        <v>68204</v>
+      </c>
+      <c r="D17" t="n">
+        <v>60</v>
+      </c>
+      <c r="E17" t="n">
+        <v>52</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1233.9</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1067</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.5735</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:O17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6283,7 +6673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6519,7 +6909,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>0</v>
       </c>
@@ -6537,8 +6926,113 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1403</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>649.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>624</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3165</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>755.8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>612</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O4"/>
+  <autoFilter ref="A1:O6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6549,7 +7043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10092,8 +10586,122 @@
         <v>0</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>166</v>
+      </c>
+      <c r="C68" t="n">
+        <v>171998</v>
+      </c>
+      <c r="D68" t="n">
+        <v>198</v>
+      </c>
+      <c r="E68" t="n">
+        <v>53</v>
+      </c>
+      <c r="F68" t="n">
+        <v>740</v>
+      </c>
+      <c r="G68" t="n">
+        <v>914</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.8245</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>SCP個別オブジェクト</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>財団組織・職員</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>15</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>167</v>
+      </c>
+      <c r="C69" t="n">
+        <v>174886</v>
+      </c>
+      <c r="D69" t="n">
+        <v>201</v>
+      </c>
+      <c r="E69" t="n">
+        <v>55</v>
+      </c>
+      <c r="F69" t="n">
+        <v>739.2</v>
+      </c>
+      <c r="G69" t="n">
+        <v>918</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.7877</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>SCP個別オブジェクト</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>財団組織・職員</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>15</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O67"/>
+  <autoFilter ref="A1:O69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10104,7 +10712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12301,7 +12909,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="n">
         <v>0</v>
       </c>
@@ -12319,8 +12926,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12331,7 +13025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14555,7 +15249,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="n">
         <v>7</v>
       </c>
@@ -14573,8 +15266,113 @@
         <v>0</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>29</v>
+      </c>
+      <c r="C47" t="n">
+        <v>58790</v>
+      </c>
+      <c r="D47" t="n">
+        <v>63</v>
+      </c>
+      <c r="E47" t="n">
+        <v>43</v>
+      </c>
+      <c r="F47" t="n">
+        <v>644.6</v>
+      </c>
+      <c r="G47" t="n">
+        <v>752</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.7606000000000001</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
+        <v>7</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>29</v>
+      </c>
+      <c r="C48" t="n">
+        <v>59410</v>
+      </c>
+      <c r="D48" t="n">
+        <v>66</v>
+      </c>
+      <c r="E48" t="n">
+        <v>45</v>
+      </c>
+      <c r="F48" t="n">
+        <v>600.7</v>
+      </c>
+      <c r="G48" t="n">
+        <v>664</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.7393</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>7</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14585,7 +15383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16346,7 +17144,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
         <v>0</v>
       </c>
@@ -16364,8 +17161,113 @@
         <v>0</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>9</v>
+      </c>
+      <c r="C37" t="n">
+        <v>47449</v>
+      </c>
+      <c r="D37" t="n">
+        <v>51</v>
+      </c>
+      <c r="E37" t="n">
+        <v>38</v>
+      </c>
+      <c r="F37" t="n">
+        <v>866.4</v>
+      </c>
+      <c r="G37" t="n">
+        <v>934</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.1822</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>9</v>
+      </c>
+      <c r="C38" t="n">
+        <v>47449</v>
+      </c>
+      <c r="D38" t="n">
+        <v>51</v>
+      </c>
+      <c r="E38" t="n">
+        <v>36</v>
+      </c>
+      <c r="F38" t="n">
+        <v>863.2</v>
+      </c>
+      <c r="G38" t="n">
+        <v>934</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.1931</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O36"/>
+  <autoFilter ref="A1:O38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16376,7 +17278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17606,7 +18508,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>0</v>
       </c>
@@ -17624,8 +18525,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O26"/>
+  <autoFilter ref="A1:O28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17636,7 +18624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18359,7 +19347,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -18377,8 +19364,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:O17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18389,7 +19463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19102,7 +20176,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -19120,8 +20193,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:O17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19132,7 +20292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19845,7 +21005,6 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -19863,8 +21022,95 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:O17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>